<commit_message>
feat: reply body preview in modal + clean RFC822 parsing + Envoyés count fix
</commit_message>
<xml_diff>
--- a/TEST_new.xlsx
+++ b/TEST_new.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexcohenskalli/Documents/PERSO/Gavroch.dev/Gavroch.dev/hatmada/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C9DBA20-972E-7B4D-9AD7-DCEDDAD59CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5B9B93-1686-0442-A6B7-1FF8D8CEBB28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{6748F77D-2A60-DC47-8FB3-BA892948F9D5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Cohen-Skalli</t>
   </si>
@@ -71,19 +71,10 @@
     <t>Carrefour</t>
   </si>
   <si>
-    <t>carrefour.com</t>
-  </si>
-  <si>
     <t>Alexandre</t>
   </si>
   <si>
-    <t>ssss</t>
-  </si>
-  <si>
     <t>alexandre.cohen-skalli@dauphine.eu</t>
-  </si>
-  <si>
-    <t>alexcoh07@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -527,7 +518,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
@@ -539,36 +530,15 @@
         <v>10</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>11</v>
-      </c>
+      <c r="E3" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{904399F0-8935-3144-B345-779A0930DB70}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{F8654E8B-C2D6-A64C-BA70-C69AEF3EB8C2}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{2C3B2232-4C7A-3746-B67D-19C7931F9265}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Migration vers GPT-4o-mini, système d'approbation d'utilisateurs et correction du bug de détection de réponses
- Remplacé Claude (Anthropic) par OpenAI GPT-4o-mini pour la génération d'emails
- Implémenté système d'approbation admin pour les nouveaux comptes
- Créé endpoint admin /api/admin/users pour gérer les approbations
- Créé page dashboard admin /dashboard/admin/users
- Corrigé bug critique dans la détection de réponses (chronologie des dates)
- Migré vers SQLite pour développement local (simplifié)
- Créé singleton Prisma en lib/prisma.ts
- Downgrade Prisma 6.2.0 pour compatibilité SQLite
- Suppression de tous les templates d'emails codés en dur
</commit_message>
<xml_diff>
--- a/TEST_new.xlsx
+++ b/TEST_new.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexcohenskalli/Documents/PERSO/Gavroch.dev/Gavroch.dev/hatmada/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5B9B93-1686-0442-A6B7-1FF8D8CEBB28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A96FA75-0CF0-CF4E-9592-C256E238807F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{6748F77D-2A60-DC47-8FB3-BA892948F9D5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>Cohen-Skalli</t>
   </si>
@@ -75,6 +75,42 @@
   </si>
   <si>
     <t>alexandre.cohen-skalli@dauphine.eu</t>
+  </si>
+  <si>
+    <t>Directrice</t>
+  </si>
+  <si>
+    <t>c'est le long</t>
+  </si>
+  <si>
+    <t>serena.skalli@gmail.com</t>
+  </si>
+  <si>
+    <t>Serena</t>
+  </si>
+  <si>
+    <t>Raphael</t>
+  </si>
+  <si>
+    <t>Directeur</t>
+  </si>
+  <si>
+    <t>ta gueule</t>
+  </si>
+  <si>
+    <t>raphael.c.skalli@gmail.com</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Directeur Export </t>
+  </si>
+  <si>
+    <t>Babyliss</t>
+  </si>
+  <si>
+    <t>david.c.skalli@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -480,11 +516,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A563101B-6783-A54F-84CC-271BE425E01E}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -534,11 +570,62 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E3" s="1"/>
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{2C3B2232-4C7A-3746-B67D-19C7931F9265}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{F41BBDB0-E4CC-9349-B453-B2984596BA83}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{AD4FDD3E-BA59-C146-9214-46A202E5BF96}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{ED06B65A-A143-004B-8A60-734F562AE54B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>